<commit_message>
feat: Enhance IWA AI and property handling in XLSX processing
Signed-off-by: gayanath8 <gayanathr@xeptagon.com>
</commit_message>
<xml_diff>
--- a/guardian-service/artifacts/template.xlsx
+++ b/guardian-service/artifacts/template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="231">
   <si>
     <t xml:space="preserve">  Guardian Schema Template</t>
   </si>
@@ -490,6 +490,12 @@
   </si>
   <si>
     <t>A geo field's Parameter must hold the key of a legal parent field: a Country may point at a Continent, a State/Province at a Country. A key that matches no field in the schema, or an illegal pairing, is a row-level import error.</t>
+  </si>
+  <si>
+    <t>An unrecognized "IWA Version" value (not V1, V3, 1.0.0 or 3.0.0) is treated as V1, with a warning.</t>
+  </si>
+  <si>
+    <t>An "IWA Property" path not found in the current IWA Version's property list still imports. Guardian keeps the value and reports a warning.</t>
   </si>
   <si>
     <t>Schema name</t>
@@ -1767,7 +1773,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2641,8 +2647,26 @@
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
     </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B95" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="C95" s="28"/>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="B96" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="C96" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="43">
+  <mergeCells count="45">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A3:C3"/>
@@ -2686,6 +2710,8 @@
     <mergeCell ref="B92:C92"/>
     <mergeCell ref="B93:C93"/>
     <mergeCell ref="A94:C94"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2713,7 +2739,7 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -2730,7 +2756,7 @@
         <v>40</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C2" s="30"/>
       <c r="D2" s="30"/>
@@ -2743,10 +2769,10 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="32" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C3" s="30"/>
       <c r="D3" s="30"/>
@@ -2797,17 +2823,17 @@
         <v>96</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D5" s="35"/>
       <c r="E5" s="35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F5" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H5" s="35"/>
       <c r="I5" s="35"/>
@@ -2823,7 +2849,7 @@
       <c r="C6" s="35"/>
       <c r="D6" s="35"/>
       <c r="E6" s="35" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F6" s="35" t="s">
         <v>11</v>
@@ -2845,7 +2871,7 @@
       <c r="C7" s="35"/>
       <c r="D7" s="35"/>
       <c r="E7" s="35" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F7" s="35" t="s">
         <v>8</v>
@@ -2867,13 +2893,13 @@
       <c r="C8" s="35"/>
       <c r="D8" s="35"/>
       <c r="E8" s="35" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F8" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G8" s="35" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
@@ -2887,11 +2913,11 @@
         <v>87</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D9" s="35"/>
       <c r="E9" s="35" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F9" s="35" t="s">
         <v>8</v>
@@ -2913,7 +2939,7 @@
       <c r="C10" s="35"/>
       <c r="D10" s="35"/>
       <c r="E10" s="35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F10" s="35" t="s">
         <v>8</v>
@@ -2935,13 +2961,13 @@
       <c r="C11" s="35"/>
       <c r="D11" s="35"/>
       <c r="E11" s="35" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F11" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H11" s="35"/>
       <c r="I11" s="35"/>
@@ -2957,13 +2983,13 @@
       <c r="C12" s="35"/>
       <c r="D12" s="35"/>
       <c r="E12" s="35" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F12" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H12" s="35"/>
       <c r="I12" s="35"/>
@@ -2979,13 +3005,13 @@
       <c r="C13" s="35"/>
       <c r="D13" s="35"/>
       <c r="E13" s="35" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F13" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H13" s="35"/>
       <c r="I13" s="35"/>
@@ -3001,13 +3027,13 @@
       <c r="C14" s="35"/>
       <c r="D14" s="35"/>
       <c r="E14" s="35" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F14" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G14" s="35" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H14" s="35"/>
       <c r="I14" s="35"/>
@@ -3023,13 +3049,13 @@
       <c r="C15" s="35"/>
       <c r="D15" s="35"/>
       <c r="E15" s="35" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F15" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G15" s="35" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H15" s="35"/>
       <c r="I15" s="35"/>
@@ -3045,13 +3071,13 @@
       <c r="C16" s="35"/>
       <c r="D16" s="35"/>
       <c r="E16" s="35" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F16" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G16" s="35" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H16" s="35"/>
       <c r="I16" s="35"/>
@@ -3067,13 +3093,13 @@
       <c r="C17" s="35"/>
       <c r="D17" s="35"/>
       <c r="E17" s="35" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F17" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G17" s="35" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
@@ -3089,13 +3115,13 @@
       <c r="C18" s="35"/>
       <c r="D18" s="35"/>
       <c r="E18" s="35" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F18" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
@@ -3109,11 +3135,11 @@
         <v>105</v>
       </c>
       <c r="C19" s="35" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D19" s="35"/>
       <c r="E19" s="35" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F19" s="35" t="s">
         <v>8</v>
@@ -3133,7 +3159,7 @@
       <c r="C20" s="35"/>
       <c r="D20" s="36"/>
       <c r="E20" s="37" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F20" s="35" t="s">
         <v>8</v>
@@ -3151,11 +3177,11 @@
         <v>90</v>
       </c>
       <c r="C21" s="39" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D21" s="35"/>
       <c r="E21" s="35" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F21" s="35" t="s">
         <v>8</v>
@@ -3175,11 +3201,11 @@
         <v>93</v>
       </c>
       <c r="C22" s="39" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D22" s="35"/>
       <c r="E22" s="35" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F22" s="35" t="s">
         <v>8</v>
@@ -3201,13 +3227,13 @@
       <c r="C23" s="35"/>
       <c r="D23" s="38"/>
       <c r="E23" s="37" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F23" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G23" s="35" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="H23" s="35"/>
       <c r="I23" s="35"/>
@@ -3221,11 +3247,11 @@
         <v>108</v>
       </c>
       <c r="C24" s="35" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D24" s="38"/>
       <c r="E24" s="37" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F24" s="35" t="s">
         <v>8</v>
@@ -3234,7 +3260,7 @@
       <c r="H24" s="35"/>
       <c r="I24" s="35"/>
       <c r="J24" s="35" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -3247,18 +3273,18 @@
       <c r="C25" s="35"/>
       <c r="D25" s="38"/>
       <c r="E25" s="37" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F25" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G25" s="35" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H25" s="35"/>
       <c r="I25" s="35"/>
       <c r="J25" s="35" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -3271,18 +3297,18 @@
       <c r="C26" s="35"/>
       <c r="D26" s="38"/>
       <c r="E26" s="37" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F26" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G26" s="35" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H26" s="35"/>
       <c r="I26" s="35"/>
       <c r="J26" s="35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -3293,22 +3319,22 @@
         <v>115</v>
       </c>
       <c r="C27" s="35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D27" s="38"/>
       <c r="E27" s="37" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F27" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G27" s="35" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H27" s="35"/>
       <c r="I27" s="35"/>
       <c r="J27" s="35" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -3319,25 +3345,25 @@
         <v>118</v>
       </c>
       <c r="C28" s="35" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D28" s="38"/>
       <c r="E28" s="37" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F28" s="35" t="s">
         <v>8</v>
       </c>
       <c r="G28" s="35" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H28" s="35"/>
       <c r="I28" s="35"/>
       <c r="J28" s="35" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="29" collapsed="1" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="38" t="s">
         <v>8</v>
       </c>
@@ -3349,19 +3375,19 @@
         <f>EXACT(G5,"Option 1")</f>
       </c>
       <c r="E29" s="42" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F29" s="37" t="s">
         <v>8</v>
       </c>
       <c r="G29" s="35" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H29" s="35"/>
       <c r="I29" s="35"/>
       <c r="J29" s="35"/>
     </row>
-    <row r="30" collapsed="1" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
         <v>8</v>
       </c>
@@ -3373,13 +3399,13 @@
         <f>NOT(EXACT(G5,"Option 1"))</f>
       </c>
       <c r="E30" s="42" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F30" s="42" t="s">
         <v>8</v>
       </c>
       <c r="G30" s="42" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H30" s="42"/>
       <c r="I30" s="42"/>
@@ -3397,13 +3423,13 @@
         <v>8</v>
       </c>
       <c r="E31" s="44" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F31" s="44" t="s">
         <v>8</v>
       </c>
       <c r="G31" s="44" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H31" s="44"/>
       <c r="I31" s="44"/>
@@ -3417,11 +3443,11 @@
         <v>102</v>
       </c>
       <c r="C32" s="44" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D32" s="45"/>
       <c r="E32" s="44" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F32" s="44" t="s">
         <v>8</v>
@@ -3441,11 +3467,11 @@
         <v>99</v>
       </c>
       <c r="C33" s="44" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D33" s="45"/>
       <c r="E33" s="44" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F33" s="44" t="s">
         <v>8</v>
@@ -3465,13 +3491,13 @@
       <c r="C34" s="47"/>
       <c r="D34" s="48"/>
       <c r="E34" s="47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F34" s="47" t="s">
         <v>8</v>
       </c>
       <c r="G34" s="47" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H34" s="47"/>
       <c r="I34" s="47"/>
@@ -3487,7 +3513,7 @@
       <c r="C35" s="47"/>
       <c r="D35" s="48"/>
       <c r="E35" s="47" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F35" s="47" t="s">
         <v>11</v>
@@ -3507,11 +3533,11 @@
         <v>99</v>
       </c>
       <c r="C36" s="49" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D36" s="45"/>
       <c r="E36" s="44" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F36" s="44" t="s">
         <v>8</v>
@@ -3531,13 +3557,13 @@
       <c r="C37" s="47"/>
       <c r="D37" s="48"/>
       <c r="E37" s="47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F37" s="47" t="s">
         <v>8</v>
       </c>
       <c r="G37" s="47" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H37" s="47"/>
       <c r="I37" s="47"/>
@@ -3553,7 +3579,7 @@
       <c r="C38" s="47"/>
       <c r="D38" s="48"/>
       <c r="E38" s="47" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F38" s="47" t="s">
         <v>11</v>
@@ -3573,11 +3599,11 @@
         <v>99</v>
       </c>
       <c r="C39" s="49" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D39" s="45"/>
       <c r="E39" s="44" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F39" s="44" t="s">
         <v>8</v>
@@ -3597,13 +3623,13 @@
       <c r="C40" s="47"/>
       <c r="D40" s="48"/>
       <c r="E40" s="47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F40" s="47" t="s">
         <v>8</v>
       </c>
       <c r="G40" s="47" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H40" s="47"/>
       <c r="I40" s="47"/>
@@ -3617,11 +3643,11 @@
         <v>96</v>
       </c>
       <c r="C41" s="47" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D41" s="48"/>
       <c r="E41" s="47" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F41" s="47"/>
       <c r="G41" s="47"/>
@@ -3637,11 +3663,11 @@
         <v>99</v>
       </c>
       <c r="C42" s="49" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D42" s="45"/>
       <c r="E42" s="44" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F42" s="44" t="s">
         <v>8</v>
@@ -3651,7 +3677,7 @@
       <c r="I42" s="44"/>
       <c r="J42" s="44"/>
     </row>
-    <row r="43" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25" outlineLevel="2">
+    <row r="43" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25" outlineLevel="2" collapsed="1">
       <c r="A43" s="46" t="s">
         <v>8</v>
       </c>
@@ -3661,19 +3687,19 @@
       <c r="C43" s="47"/>
       <c r="D43" s="48"/>
       <c r="E43" s="47" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F43" s="47" t="s">
         <v>8</v>
       </c>
       <c r="G43" s="47" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H43" s="47"/>
       <c r="I43" s="47"/>
       <c r="J43" s="47"/>
     </row>
-    <row r="44" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25" outlineLevel="2">
+    <row r="44" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25" outlineLevel="2" collapsed="1">
       <c r="A44" s="50" t="s">
         <v>11</v>
       </c>
@@ -3683,7 +3709,7 @@
       <c r="C44" s="51"/>
       <c r="D44" s="52"/>
       <c r="E44" s="51" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F44" s="51" t="s">
         <v>11</v>
@@ -3719,7 +3745,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3727,61 +3753,61 @@
     <col min="3" max="3" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="17" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="53" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B1" s="53" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C1" s="53" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="54" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B2" s="54" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="54"/>
       <c r="B3" s="54"/>
       <c r="C3" s="54" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="54"/>
       <c r="B4" s="54"/>
       <c r="C4" s="54" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="54" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B5" s="54" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="54" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="54"/>
       <c r="B6" s="54"/>
       <c r="C6" s="54" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="54"/>
       <c r="B7" s="54"/>
       <c r="C7" s="54"/>

</xml_diff>